<commit_message>
finalized clusters - lots of time wasted
</commit_message>
<xml_diff>
--- a/data-files/0-final-analysis/0-summary/exploratory_analysis_findings.xlsx
+++ b/data-files/0-final-analysis/0-summary/exploratory_analysis_findings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://envienstudio.sharepoint.com/Shared Documents/Potential/DOE RD Submission/3 - Market Research/doe-SBIR-research-project/data-files/0-final-analysis/0-summary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="143" documentId="8_{429CFAF0-D855-478C-922B-46BC6034CCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59D028F0-9F8E-4F9B-A7F1-5A44BE46C434}"/>
+  <xr:revisionPtr revIDLastSave="145" documentId="8_{429CFAF0-D855-478C-922B-46BC6034CCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E9BD71B-11C8-4714-A0D3-E5634D01175D}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{F90B1637-CABF-4440-8D8C-4382C5054209}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F90B1637-CABF-4440-8D8C-4382C5054209}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -447,7 +447,7 @@
     <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -41036,9 +41036,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -41076,7 +41076,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -41182,7 +41182,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -41324,7 +41324,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -42284,15 +42284,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005983132403D1464F8DDC272820BA8C1B" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6fe6f55e11da51139aa85f6a00701c7d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d4fe9914-c092-4200-a7d8-cc85a6bef288" xmlns:ns3="afc29c3b-9522-4360-ba9d-c1dc5ac90a19" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="285f550d8d1fc9956465dc5fad4d328f" ns2:_="" ns3:_="">
     <xsd:import namespace="d4fe9914-c092-4200-a7d8-cc85a6bef288"/>
@@ -42541,6 +42532,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -42553,14 +42553,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{739ADEE7-F8A3-42DF-98B7-EB01FBFBB8B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6594A5B1-E02F-47EE-BAEB-D1609F1F608D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -42579,6 +42571,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{739ADEE7-F8A3-42DF-98B7-EB01FBFBB8B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE09E3A6-313E-4615-A55C-D77C33A5384B}">
   <ds:schemaRefs>

</xml_diff>